<commit_message>
Added output argument logic in sheet2dbo file
</commit_message>
<xml_diff>
--- a/bos-onboarding/test/jinesh1.xlsx
+++ b/bos-onboarding/test/jinesh1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\GitHub\SDIOTECS_IN_BLR_ANANTA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\build2auto\bos-tools\bos-onboarding\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF9571F-6659-46BE-8DE7-22091F646591}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2EA58C-6594-418B-913F-1B45A6899C5D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>